<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@5f4337013a9b23ab9c8fd2ad1cd02099a66d3811 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-ICPC-1-NL.xlsx
+++ b/CodeSystem-ICPC-1-NL.xlsx
@@ -29,7 +29,7 @@
     <t>Identifier</t>
   </si>
   <si>
-    <t>id: Uniform Resource Identifier (URI)#urn:oid:2.16.840.1.113883.2.4.4.31.1</t>
+    <t>urn:ietf:rfc:3986#Uniform Resource Identifier (URI)#urn:oid:2.16.840.1.113883.2.4.4.31.1</t>
   </si>
   <si>
     <t>Version</t>
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-01-29T15:53:55+00:00</t>
+    <t>2024-01-31T09:56:58+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@979760976d73125f008303352e158c9e6988e990 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-ICPC-1-NL.xlsx
+++ b/CodeSystem-ICPC-1-NL.xlsx
@@ -35,7 +35,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.20.0</t>
+    <t>0.21.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-02-15T10:45:28+00:00</t>
+    <t>2024-02-16T07:23:31+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@42c236eb67d208341153bd93bb848f6e67a8c5f2 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-ICPC-1-NL.xlsx
+++ b/CodeSystem-ICPC-1-NL.xlsx
@@ -35,7 +35,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.21.0</t>
+    <t>0.22.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-02-21T07:49:13+00:00</t>
+    <t>2024-02-21T07:54:13+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@589de11e060d8f4358c44606c88c3db12b68ba51 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-ICPC-1-NL.xlsx
+++ b/CodeSystem-ICPC-1-NL.xlsx
@@ -35,7 +35,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.22.0</t>
+    <t>0.23.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-03-04T08:09:52+00:00</t>
+    <t>2024-03-04T08:15:04+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@12ae779ba3a045dfb63331a0f0ce65e2997f0f2d 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-ICPC-1-NL.xlsx
+++ b/CodeSystem-ICPC-1-NL.xlsx
@@ -35,7 +35,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.23.0</t>
+    <t>0.24.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-03-18T14:33:52+00:00</t>
+    <t>2024-03-19T08:53:44+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@1353becf10db20f3ec192d0d7df1e17217a3f3f8 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-ICPC-1-NL.xlsx
+++ b/CodeSystem-ICPC-1-NL.xlsx
@@ -29,7 +29,7 @@
     <t>Identifier</t>
   </si>
   <si>
-    <t>urn:ietf:rfc:3986#Uniform Resource Identifier (URI)#urn:oid:2.16.840.1.113883.2.4.4.31.1</t>
+    <t>OID:2.16.840.1.113883.2.4.4.31.1</t>
   </si>
   <si>
     <t>Version</t>
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-03-19T08:53:44+00:00</t>
+    <t>2024-03-20T18:23:37+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@49c8771f78c39e0b74a7e650e7711fc5ca4c86b2 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-ICPC-1-NL.xlsx
+++ b/CodeSystem-ICPC-1-NL.xlsx
@@ -35,7 +35,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.24.0</t>
+    <t>0.25.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-04-26T06:40:39+00:00</t>
+    <t>2024-04-26T10:53:01+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@2c46a51a9e256b4bb0a30b8b4e4c647c010f3a42 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-ICPC-1-NL.xlsx
+++ b/CodeSystem-ICPC-1-NL.xlsx
@@ -35,7 +35,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.25.0</t>
+    <t>0.26.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-05-13T07:39:20+00:00</t>
+    <t>2024-05-13T07:45:44+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@4a53dc85c5409e5ce60bb7a3eb1e488d6bc76e72 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-ICPC-1-NL.xlsx
+++ b/CodeSystem-ICPC-1-NL.xlsx
@@ -35,7 +35,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.26.0</t>
+    <t>0.27.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-05-29T07:17:54+00:00</t>
+    <t>2024-05-29T07:26:47+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@5dac0ae24f82765f53ea0108c1c09e489af8a204 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-ICPC-1-NL.xlsx
+++ b/CodeSystem-ICPC-1-NL.xlsx
@@ -35,7 +35,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.27.0</t>
+    <t>1.2.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-06-21T09:41:55+00:00</t>
+    <t>2024-06-21T10:00:31+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@2b1316e4405e306e1e7ca3eed156ed615a07f989 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-ICPC-1-NL.xlsx
+++ b/CodeSystem-ICPC-1-NL.xlsx
@@ -35,7 +35,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.2.0</t>
+    <t>1.3.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-07-26T10:44:53+00:00</t>
+    <t>2024-07-26T10:53:24+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@d9cfd2a5d9315aa02cbbc129b2cbd041459adc68 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-ICPC-1-NL.xlsx
+++ b/CodeSystem-ICPC-1-NL.xlsx
@@ -35,7 +35,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.3.0</t>
+    <t>1.4.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-08-06T13:05:08+00:00</t>
+    <t>2024-08-06T13:09:13+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@c8b7eede9f749186ec729aed0c41594262e23c11 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-ICPC-1-NL.xlsx
+++ b/CodeSystem-ICPC-1-NL.xlsx
@@ -35,7 +35,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.4.0</t>
+    <t>1.5.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-08-23T11:18:20+00:00</t>
+    <t>2024-08-23T11:22:37+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@07f4c956fffc014d03f31c1368abd34fd012e062 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-ICPC-1-NL.xlsx
+++ b/CodeSystem-ICPC-1-NL.xlsx
@@ -35,7 +35,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.5.0</t>
+    <t>1.6.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-09-30T11:48:36+00:00</t>
+    <t>2024-09-30T11:54:02+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@20d37dec720bac99174ab02ac06fbceb13d5de51 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-ICPC-1-NL.xlsx
+++ b/CodeSystem-ICPC-1-NL.xlsx
@@ -35,7 +35,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.6.0</t>
+    <t>1.7.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-10-17T08:27:04+00:00</t>
+    <t>2024-10-17T08:35:21+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@62757800ffbdf2ece08ff11cf76d294e30523652 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-ICPC-1-NL.xlsx
+++ b/CodeSystem-ICPC-1-NL.xlsx
@@ -35,7 +35,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.7.0</t>
+    <t>1.8.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-11-12T08:18:00+00:00</t>
+    <t>2024-11-12T08:24:06+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@cf7e18cdedf335ebbc166900d1978f86214e2f42 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-ICPC-1-NL.xlsx
+++ b/CodeSystem-ICPC-1-NL.xlsx
@@ -35,7 +35,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.8.0</t>
+    <t>1.9.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-11-25T09:37:54+00:00</t>
+    <t>2024-11-25T09:42:11+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@aa14b4bfbc9e0befc7ee597bbf503989c164bca8 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-ICPC-1-NL.xlsx
+++ b/CodeSystem-ICPC-1-NL.xlsx
@@ -35,7 +35,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.9.0</t>
+    <t>1.10.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-12-10T08:19:29+00:00</t>
+    <t>2024-12-10T08:34:20+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@23bd9178259a7e0a3cf09e09c06b819c3b3bee9f 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-ICPC-1-NL.xlsx
+++ b/CodeSystem-ICPC-1-NL.xlsx
@@ -35,7 +35,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.10.0</t>
+    <t>1.11.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-12-27T09:59:08+00:00</t>
+    <t>2025-01-02T11:11:09+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@81776909ce83feee5dad1e04e4836a8deb0570bf 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-ICPC-1-NL.xlsx
+++ b/CodeSystem-ICPC-1-NL.xlsx
@@ -35,7 +35,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.11.0</t>
+    <t>1.12.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-01-28T20:06:40+00:00</t>
+    <t>2025-01-28T20:08:20+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>